<commit_message>
Workbook: quote Q2 2026 call guidance in six text cells
Replace only the text of six shared strings in CAT_8Q_Operating_Dataset.xlsx
(Dealer Inventory!D11, Source Index!D16 and D24, Comparability Log!F18,
Analysis!A60 and A63) so the workbook matches the attributed public wording.
D11 now quotes the Q2 call sentence exactly, without "about". Every other
entry in the .xlsx package is byte-identical; formulas, cached values and
the 32 cached reconciliation zeros are unchanged. DEFERRED.md marks the
drawdown and FY2026 tariff-guidance evidence gaps resolved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UruoBzZjv6K37Wc7Y22YbC
</commit_message>
<xml_diff>
--- a/caterpillar-demand-quality/model/CAT_8Q_Operating_Dataset.xlsx
+++ b/caterpillar-demand-quality/model/CAT_8Q_Operating_Dataset.xlsx
@@ -362,7 +362,7 @@
     <t xml:space="preserve">G-H are the disclosed unfavorable CI manufacturing-cost figures (SOURCED). Caterpillar said they 'largely reflected' higher tariff costs, so treating them as the full tariff effect is an approximation. I is the 340 bps disclosed on the Q2 2026 call (CFO Kyle Epley, SOURCED), converted to about $284M here (DERIVED). G-H and I use different methods; do not read them as a trend.</t>
   </si>
   <si>
-    <t xml:space="preserve">READ (INTERPRETIVE): Q4 2025 reported 14.9% is the series low; ex-tariff it sits near 20.9%, inside the 19.6-20.4% band of the surrounding quarters. Our reading is that the trough was mainly a tariff cost shock rather than demand or execution; manufacturing costs are not purely tariffs, and the Q4 2025 profit bridge leaves a $14M unitemized residual. It is NOT one-time: tariffs recur while in force. CI was still carrying about 509 bps (workbook method) in Q1 2026 and 340 bps (disclosed) in Q2 2026. Q3 2026 CI tariff guidance: INSUFFICIENT EVIDENCE (no verbatim quote captured).</t>
+    <t xml:space="preserve">READ (INTERPRETIVE): Q4 2025 reported 14.9% is the series low; ex-tariff it sits near 20.9%, inside the 19.6-20.4% band of the surrounding quarters. Our reading is that the trough was mainly a tariff cost shock rather than demand or execution; manufacturing costs are not purely tariffs, and the Q4 2025 profit bridge leaves a $14M unitemized residual. It is NOT one-time: tariffs recur while in force. CI was still carrying about 509 bps (workbook method) in Q1 2026 and 340 bps (disclosed) in Q2 2026. For Q3 2026, management expects tariff costs of around $600 million with about 50% incurred in Construction Industries (CFO Kyle Epley, Q2 2026 call).</t>
   </si>
   <si>
     <t xml:space="preserve">EX-TARIFF SEQUENCE: about 20.9% -&gt; 26.5% -&gt; 26.7%. Reported moves 14.9% -&gt; 21.4% -&gt; 23.3% (SOURCED), about 840 bps (DERIVED; +/-10 bps from one-decimal rounding). Lower tariff pressure and volume leverage with price realization both contributed (INTERPRETIVE), but the disclosures do not support a consistent split.</t>
@@ -371,7 +371,7 @@
     <t xml:space="preserve">CAVEAT — do not read ex-tariff margin as underlying performance. Price realization swung from -$60M to +$356M to +$309M largely to RECOVER tariffs. Removing the tariff cost while keeping the price taken to offset it double-counts the benefit. Ex-tariff margin is therefore an UPPER BOUND on underlying improvement. The cleanest genuine component is volume leverage.</t>
   </si>
   <si>
-    <t xml:space="preserve">IEEPA RECOVERIES: Q2 2026 operating profit included $392M of expected IEEPA tariff recoveries (SOURCED). CFO Kyle Epley stated "the majority of this amount reflected in corporate items" (SOURCED). The CI share was not disclosed, so CI segment margin (23.3%) is unlikely to be materially affected; that is an INFERENCE, not a confirmed exclusion. The recovery IS one-time; the tariff costs are not. FY2026 tariff cost guidance (about $2.2B): INSUFFICIENT EVIDENCE (no verbatim quote captured).</t>
+    <t xml:space="preserve">IEEPA RECOVERIES: Q2 2026 operating profit included $392M of expected IEEPA tariff recoveries (SOURCED). CFO Kyle Epley stated "the majority of this amount reflected in corporate items" (SOURCED). The CI share was not disclosed, so CI segment margin (23.3%) is unlikely to be materially affected; that is an INFERENCE, not a confirmed exclusion. The recovery IS one-time; the tariff costs are not. Management expects full-year 2026 tariff costs of around $2.2 billion, excluding approximately $400 million of expected IEEPA tariff recoveries, at the low end of its prior range (CFO Kyle Epley, Q2 2026 call).</t>
   </si>
   <si>
     <t xml:space="preserve">HEADLINE: Q4 2025 CI reported margin 14.9%, tariff-related drag ~604 bps (workbook method). Q1 2026 ~509 bps (workbook method). Q2 2026 340 bps (disclosed on the call). Ex-tariff: ~20.9% / ~26.5% / ~26.7% (upper bound, see row 62).</t>
@@ -620,7 +620,7 @@
     <t xml:space="preserve">CI only</t>
   </si>
   <si>
-    <t xml:space="preserve">10-Q: "Construction Industries dealer inventory increased by $400 million"  |  Call (corroborating): "Dealer inventory increased by about $400 million in Construction Industries."</t>
+    <t xml:space="preserve">10-Q: "Construction Industries dealer inventory increased by $400 million"  |  Call (corroborating): "Dealer inventory increased by $400 million in Construction Industries compared to a decrease in the second quarter of 2025."</t>
   </si>
   <si>
     <t xml:space="preserve">Q2 2026 Form 10-Q, Item 2 MD&amp;A — accession 0000018230-26-000046; corroborated by Q2 2026 earnings call</t>
@@ -1016,7 +1016,7 @@
     <t xml:space="preserve">Our reading (INTERPRETIVE): reported CI margin of 14.9% in Q4 2025 was mainly a tariff cost shock rather than demand weakness or operating deterioration; the disclosed manufacturing costs only 'largely' reflected tariffs. Ex-tariff it sits near 20.9%, inside the 19.6-20.4% band of the surrounding quarters. Using the reported series as a baseline overstates the 2026 recovery.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ex-tariff margin shown on the Analysis tab for all three quarters (Q2 2026 on a different method). NOT a one-time item: tariffs recur while in force. FY2026 tariff guidance (about $2.2bn, roughly half of Q3 in CI) was recorded without a verbatim quote: INSUFFICIENT EVIDENCE, not used in the analysis.</t>
+    <t xml:space="preserve">Ex-tariff margin shown on the Analysis tab for all three quarters (Q2 2026 on a different method). NOT a one-time item: tariffs recur while in force. Management expects full-year 2026 tariff costs of around $2.2 billion, excluding approximately $400 million of expected IEEPA tariff recoveries, at the low end of its prior range; for Q3 2026 it expects tariff costs of around $600 million with about 50% incurred in Construction Industries (CFO Kyle Epley, Q2 2026 call).</t>
   </si>
   <si>
     <t xml:space="preserve">16</t>
@@ -1145,7 +1145,7 @@
     <t xml:space="preserve">https://www.fool.com/earnings/call-transcripts/2026/08/11/caterpillar-cat-q2-2026-earnings-call-transcript/</t>
   </si>
   <si>
-    <t xml:space="preserve">CI dealer inventory +$400M. Q4 drawdown commentary: no verbatim quote captured, INSUFFICIENT EVIDENCE; not used as a finding.</t>
+    <t xml:space="preserve">CI dealer inventory +$400M. Q4 2026 CI dealer-inventory drawdown expected: CFO Kyle Epley, "a more typical reduction in Construction Industries dealer inventory of over $1 billion in the fourth quarter"; CEO Joseph Creed, "We'll have a drawdown in the fourth quarter on CI dealer inventory."</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.fool.com/earnings/call-transcripts/2026/04/30/caterpillar-cat-q1-2026-earnings-transcript/</t>
@@ -1190,7 +1190,7 @@
     <t xml:space="preserve">Q2 2026 Earnings Call Transcript</t>
   </si>
   <si>
-    <t xml:space="preserve">CI tariff impact 340 bps; IEEPA $392M, majority in corporate items. FY26 tariff cost ~$2.2B: no verbatim quote captured, INSUFFICIENT EVIDENCE.</t>
+    <t xml:space="preserve">CI tariff impact 340 bps; IEEPA $392M, majority in corporate items. FY2026 tariff costs expected around $2.2B, excluding approximately $400M of expected IEEPA tariff recoveries, at the low end of the prior range; Q3 2026 tariff costs expected around $600M, about 50% in CI (CFO Kyle Epley).</t>
   </si>
 </sst>
 </file>

</xml_diff>